<commit_message>
Filled datagaps in 2024-25 data with other WT data
</commit_message>
<xml_diff>
--- a/Seasonality and Trends Publication/Metadata and output results.xlsx
+++ b/Seasonality and Trends Publication/Metadata and output results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bailey.armos\projects\Temp_project\report_notebooks\dev_coastal-water-temperature\Seasonality and Trends Publication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394BED35-4426-40DC-A672-C5FAC5B75CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49DCD716-C5EC-48C3-BB5F-CACF063A6BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Station inventory" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1393" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1395" uniqueCount="275">
   <si>
     <t>geoorder</t>
   </si>
@@ -863,6 +863,9 @@
   </si>
   <si>
     <t>Peak diff shift</t>
+  </si>
+  <si>
+    <t>Difference between the peak WT month and MSL month</t>
   </si>
 </sst>
 </file>
@@ -874,7 +877,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -916,6 +919,13 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -976,7 +986,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
@@ -1046,6 +1056,7 @@
     <xf numFmtId="4" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1271,7 +1282,7 @@
   <dimension ref="A1:R96"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1355,13 +1366,13 @@
       <c r="I2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="7" t="e">
-        <f t="shared" ref="J2:J96" ca="1" si="0">_xludf.DAYS(F2,E2)</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="K2" s="8" t="e">
-        <f t="shared" ref="K2:K96" ca="1" si="1">J2/365.25</f>
-        <v>#NAME?</v>
+      <c r="J2" s="7">
+        <f>_xlfn.DAYS(F2,E2)</f>
+        <v>10285</v>
+      </c>
+      <c r="K2" s="8">
+        <f t="shared" ref="K2:K96" si="0">J2/365.25</f>
+        <v>28.158795345653662</v>
       </c>
       <c r="L2" s="7">
         <v>91.15</v>
@@ -1370,7 +1381,7 @@
         <v>9376</v>
       </c>
       <c r="N2" s="9">
-        <f t="shared" ref="N2:N96" si="2">M2/365.25</f>
+        <f t="shared" ref="N2:N96" si="1">M2/365.25</f>
         <v>25.670088980150581</v>
       </c>
       <c r="O2" s="10">
@@ -1414,13 +1425,13 @@
       <c r="I3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K3" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J3" s="7">
+        <f t="shared" ref="J3:J66" si="2">_xlfn.DAYS(F3,E3)</f>
+        <v>8970</v>
+      </c>
+      <c r="K3" s="8">
+        <f t="shared" si="0"/>
+        <v>24.558521560574949</v>
       </c>
       <c r="L3" s="7">
         <v>83.43</v>
@@ -1429,7 +1440,7 @@
         <v>7475</v>
       </c>
       <c r="N3" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>20.465434633812457</v>
       </c>
       <c r="O3" s="10">
@@ -1473,13 +1484,13 @@
       <c r="I4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J4" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K4" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J4" s="7">
+        <f t="shared" si="2"/>
+        <v>9594</v>
+      </c>
+      <c r="K4" s="8">
+        <f t="shared" si="0"/>
+        <v>26.266940451745381</v>
       </c>
       <c r="L4" s="7">
         <v>80.69</v>
@@ -1488,7 +1499,7 @@
         <v>7742</v>
       </c>
       <c r="N4" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.196440793976727</v>
       </c>
       <c r="O4" s="10">
@@ -1532,13 +1543,13 @@
       <c r="I5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J5" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K5" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J5" s="7">
+        <f t="shared" si="2"/>
+        <v>9320</v>
+      </c>
+      <c r="K5" s="8">
+        <f t="shared" si="0"/>
+        <v>25.516769336071185</v>
       </c>
       <c r="L5" s="7">
         <v>90.34</v>
@@ -1547,7 +1558,7 @@
         <v>8419</v>
       </c>
       <c r="N5" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>23.049965776865161</v>
       </c>
       <c r="O5" s="10">
@@ -1591,13 +1602,13 @@
       <c r="I6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K6" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J6" s="7">
+        <f t="shared" si="2"/>
+        <v>10355</v>
+      </c>
+      <c r="K6" s="8">
+        <f t="shared" si="0"/>
+        <v>28.350444900752908</v>
       </c>
       <c r="L6" s="7">
         <v>96.81</v>
@@ -1606,7 +1617,7 @@
         <v>10026</v>
       </c>
       <c r="N6" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.449691991786448</v>
       </c>
       <c r="O6" s="10">
@@ -1650,13 +1661,13 @@
       <c r="I7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K7" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J7" s="7">
+        <f t="shared" si="2"/>
+        <v>10328</v>
+      </c>
+      <c r="K7" s="8">
+        <f t="shared" si="0"/>
+        <v>28.276522929500342</v>
       </c>
       <c r="L7" s="7">
         <v>95.3</v>
@@ -1665,7 +1676,7 @@
         <v>9840</v>
       </c>
       <c r="N7" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.940451745379878</v>
       </c>
       <c r="O7" s="10">
@@ -1709,13 +1720,13 @@
       <c r="I8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K8" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J8" s="7">
+        <f t="shared" si="2"/>
+        <v>8860</v>
+      </c>
+      <c r="K8" s="8">
+        <f t="shared" si="0"/>
+        <v>24.257357973990416</v>
       </c>
       <c r="L8" s="7">
         <v>97.05</v>
@@ -1724,7 +1735,7 @@
         <v>8581</v>
       </c>
       <c r="N8" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>23.493497604380561</v>
       </c>
       <c r="O8" s="10">
@@ -1768,13 +1779,13 @@
       <c r="I9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J9" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K9" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J9" s="7">
+        <f t="shared" si="2"/>
+        <v>8858</v>
+      </c>
+      <c r="K9" s="8">
+        <f t="shared" si="0"/>
+        <v>24.251882272416154</v>
       </c>
       <c r="L9" s="7">
         <v>94.47</v>
@@ -1783,7 +1794,7 @@
         <v>8353</v>
       </c>
       <c r="N9" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>22.869267624914443</v>
       </c>
       <c r="O9" s="10">
@@ -1827,13 +1838,13 @@
       <c r="I10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J10" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K10" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J10" s="7">
+        <f t="shared" si="2"/>
+        <v>8864</v>
+      </c>
+      <c r="K10" s="8">
+        <f t="shared" si="0"/>
+        <v>24.268309377138944</v>
       </c>
       <c r="L10" s="7">
         <v>91.51</v>
@@ -1842,7 +1853,7 @@
         <v>8091</v>
       </c>
       <c r="N10" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>22.151950718685832</v>
       </c>
       <c r="O10" s="10">
@@ -1886,13 +1897,13 @@
       <c r="I11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K11" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J11" s="7">
+        <f t="shared" si="2"/>
+        <v>10341</v>
+      </c>
+      <c r="K11" s="8">
+        <f t="shared" si="0"/>
+        <v>28.312114989733061</v>
       </c>
       <c r="L11" s="7">
         <v>93.75</v>
@@ -1901,7 +1912,7 @@
         <v>9691</v>
       </c>
       <c r="N11" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.532511978097194</v>
       </c>
       <c r="O11" s="10">
@@ -1945,13 +1956,13 @@
       <c r="I12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K12" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J12" s="7">
+        <f t="shared" si="2"/>
+        <v>10455</v>
+      </c>
+      <c r="K12" s="8">
+        <f t="shared" si="0"/>
+        <v>28.624229979466119</v>
       </c>
       <c r="L12" s="7">
         <v>88.09</v>
@@ -1960,7 +1971,7 @@
         <v>9210</v>
       </c>
       <c r="N12" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.215605749486652</v>
       </c>
       <c r="O12" s="10">
@@ -2004,13 +2015,13 @@
       <c r="I13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J13" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K13" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J13" s="7">
+        <f t="shared" si="2"/>
+        <v>8908</v>
+      </c>
+      <c r="K13" s="8">
+        <f t="shared" si="0"/>
+        <v>24.388774811772759</v>
       </c>
       <c r="L13" s="7">
         <v>83.45</v>
@@ -2019,7 +2030,7 @@
         <v>7379</v>
       </c>
       <c r="N13" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>20.202600958247775</v>
       </c>
       <c r="O13" s="10">
@@ -2063,13 +2074,13 @@
       <c r="I14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K14" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J14" s="7">
+        <f t="shared" si="2"/>
+        <v>9196</v>
+      </c>
+      <c r="K14" s="8">
+        <f t="shared" si="0"/>
+        <v>25.177275838466805</v>
       </c>
       <c r="L14" s="7">
         <v>88.01</v>
@@ -2078,7 +2089,7 @@
         <v>8092</v>
       </c>
       <c r="N14" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>22.154688569472963</v>
       </c>
       <c r="O14" s="10">
@@ -2122,13 +2133,13 @@
       <c r="I15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K15" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J15" s="7">
+        <f t="shared" si="2"/>
+        <v>11001</v>
+      </c>
+      <c r="K15" s="8">
+        <f t="shared" si="0"/>
+        <v>30.119096509240247</v>
       </c>
       <c r="L15" s="7">
         <v>92.87</v>
@@ -2137,7 +2148,7 @@
         <v>10218</v>
       </c>
       <c r="N15" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.975359342915812</v>
       </c>
       <c r="O15" s="10">
@@ -2181,13 +2192,13 @@
       <c r="I16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K16" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J16" s="7">
+        <f t="shared" si="2"/>
+        <v>9209</v>
+      </c>
+      <c r="K16" s="8">
+        <f t="shared" si="0"/>
+        <v>25.212867898699521</v>
       </c>
       <c r="L16" s="7">
         <v>86.56</v>
@@ -2196,7 +2207,7 @@
         <v>7972</v>
       </c>
       <c r="N16" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.826146475017111</v>
       </c>
       <c r="O16" s="10">
@@ -2240,13 +2251,13 @@
       <c r="I17" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K17" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J17" s="7">
+        <f t="shared" si="2"/>
+        <v>10446</v>
+      </c>
+      <c r="K17" s="8">
+        <f t="shared" si="0"/>
+        <v>28.599589322381931</v>
       </c>
       <c r="L17" s="7">
         <v>94.01</v>
@@ -2255,7 +2266,7 @@
         <v>9821</v>
       </c>
       <c r="N17" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.888432580424368</v>
       </c>
       <c r="O17" s="10">
@@ -2299,13 +2310,13 @@
       <c r="I18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K18" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J18" s="7">
+        <f t="shared" si="2"/>
+        <v>8097</v>
+      </c>
+      <c r="K18" s="8">
+        <f t="shared" si="0"/>
+        <v>22.168377823408623</v>
       </c>
       <c r="L18" s="7">
         <v>97.25</v>
@@ -2314,7 +2325,7 @@
         <v>7861</v>
       </c>
       <c r="N18" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.522245037645447</v>
       </c>
       <c r="O18" s="10">
@@ -2358,13 +2369,13 @@
       <c r="I19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J19" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K19" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J19" s="7">
+        <f t="shared" si="2"/>
+        <v>7894</v>
+      </c>
+      <c r="K19" s="8">
+        <f t="shared" si="0"/>
+        <v>21.612594113620808</v>
       </c>
       <c r="L19" s="7">
         <v>97.28</v>
@@ -2373,7 +2384,7 @@
         <v>7661</v>
       </c>
       <c r="N19" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>20.974674880219027</v>
       </c>
       <c r="O19" s="10">
@@ -2417,13 +2428,13 @@
       <c r="I20" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K20" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J20" s="7">
+        <f t="shared" si="2"/>
+        <v>9704</v>
+      </c>
+      <c r="K20" s="8">
+        <f t="shared" si="0"/>
+        <v>26.56810403832991</v>
       </c>
       <c r="L20" s="7">
         <v>79.2</v>
@@ -2432,7 +2443,7 @@
         <v>7686</v>
       </c>
       <c r="N20" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.043121149897331</v>
       </c>
       <c r="O20" s="10">
@@ -2476,13 +2487,13 @@
       <c r="I21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K21" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J21" s="7">
+        <f t="shared" si="2"/>
+        <v>10978</v>
+      </c>
+      <c r="K21" s="8">
+        <f t="shared" si="0"/>
+        <v>30.056125941136209</v>
       </c>
       <c r="L21" s="7">
         <v>91.36</v>
@@ -2491,7 +2502,7 @@
         <v>10030</v>
       </c>
       <c r="N21" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.460643394934976</v>
       </c>
       <c r="O21" s="10">
@@ -2535,13 +2546,13 @@
       <c r="I22" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K22" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J22" s="7">
+        <f t="shared" si="2"/>
+        <v>9719</v>
+      </c>
+      <c r="K22" s="8">
+        <f t="shared" si="0"/>
+        <v>26.609171800136892</v>
       </c>
       <c r="L22" s="7">
         <v>95.67</v>
@@ -2550,7 +2561,7 @@
         <v>9299</v>
       </c>
       <c r="N22" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.459274469541409</v>
       </c>
       <c r="O22" s="10">
@@ -2594,13 +2605,13 @@
       <c r="I23" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J23" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K23" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J23" s="7">
+        <f t="shared" si="2"/>
+        <v>9683</v>
+      </c>
+      <c r="K23" s="8">
+        <f t="shared" si="0"/>
+        <v>26.510609171800137</v>
       </c>
       <c r="L23" s="7">
         <v>95.07</v>
@@ -2609,7 +2620,7 @@
         <v>9206</v>
       </c>
       <c r="N23" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.204654346338124</v>
       </c>
       <c r="O23" s="10">
@@ -2653,13 +2664,13 @@
       <c r="I24" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J24" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K24" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J24" s="7">
+        <f t="shared" si="2"/>
+        <v>7436</v>
+      </c>
+      <c r="K24" s="8">
+        <f t="shared" si="0"/>
+        <v>20.358658453114305</v>
       </c>
       <c r="L24" s="7">
         <v>94.29</v>
@@ -2668,7 +2679,7 @@
         <v>7006</v>
       </c>
       <c r="N24" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>19.1813826146475</v>
       </c>
       <c r="O24" s="10">
@@ -2712,13 +2723,13 @@
       <c r="I25" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J25" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K25" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J25" s="7">
+        <f t="shared" si="2"/>
+        <v>9694</v>
+      </c>
+      <c r="K25" s="8">
+        <f t="shared" si="0"/>
+        <v>26.540725530458591</v>
       </c>
       <c r="L25" s="7">
         <v>98.46</v>
@@ -2727,7 +2738,7 @@
         <v>9256</v>
       </c>
       <c r="N25" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.341546885694729</v>
       </c>
       <c r="O25" s="10">
@@ -2771,13 +2782,13 @@
       <c r="I26" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K26" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J26" s="7">
+        <f t="shared" si="2"/>
+        <v>10680</v>
+      </c>
+      <c r="K26" s="8">
+        <f t="shared" si="0"/>
+        <v>29.240246406570844</v>
       </c>
       <c r="L26" s="7">
         <v>98.27</v>
@@ -2786,7 +2797,7 @@
         <v>10495</v>
       </c>
       <c r="N26" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.733744010951405</v>
       </c>
       <c r="O26" s="10">
@@ -2830,13 +2841,13 @@
       <c r="I27" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J27" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K27" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J27" s="7">
+        <f t="shared" si="2"/>
+        <v>10534</v>
+      </c>
+      <c r="K27" s="8">
+        <f t="shared" si="0"/>
+        <v>28.840520191649556</v>
       </c>
       <c r="L27" s="7">
         <v>89.22</v>
@@ -2845,7 +2856,7 @@
         <v>9399</v>
       </c>
       <c r="N27" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.733059548254619</v>
       </c>
       <c r="O27" s="10">
@@ -2889,13 +2900,13 @@
       <c r="I28" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J28" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K28" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J28" s="7">
+        <f t="shared" si="2"/>
+        <v>10923</v>
+      </c>
+      <c r="K28" s="8">
+        <f t="shared" si="0"/>
+        <v>29.905544147843944</v>
       </c>
       <c r="L28" s="7">
         <v>94.75</v>
@@ -2904,7 +2915,7 @@
         <v>10351</v>
       </c>
       <c r="N28" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.33949349760438</v>
       </c>
       <c r="O28" s="10">
@@ -2948,13 +2959,13 @@
       <c r="I29" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J29" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K29" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J29" s="7">
+        <f t="shared" si="2"/>
+        <v>10768</v>
+      </c>
+      <c r="K29" s="8">
+        <f t="shared" si="0"/>
+        <v>29.481177275838466</v>
       </c>
       <c r="L29" s="7">
         <v>95.87</v>
@@ -2963,7 +2974,7 @@
         <v>10532</v>
       </c>
       <c r="N29" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.83504449007529</v>
       </c>
       <c r="O29" s="10">
@@ -3007,13 +3018,13 @@
       <c r="I30" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J30" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K30" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J30" s="7">
+        <f t="shared" si="2"/>
+        <v>10827</v>
+      </c>
+      <c r="K30" s="8">
+        <f t="shared" si="0"/>
+        <v>29.642710472279262</v>
       </c>
       <c r="L30" s="7">
         <v>89.64</v>
@@ -3022,7 +3033,7 @@
         <v>9706</v>
       </c>
       <c r="N30" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.573579739904176</v>
       </c>
       <c r="O30" s="10">
@@ -3066,13 +3077,13 @@
       <c r="I31" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J31" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K31" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J31" s="7">
+        <f t="shared" si="2"/>
+        <v>7271</v>
+      </c>
+      <c r="K31" s="8">
+        <f t="shared" si="0"/>
+        <v>19.906913073237508</v>
       </c>
       <c r="L31" s="7">
         <v>88.42</v>
@@ -3081,7 +3092,7 @@
         <v>6404</v>
       </c>
       <c r="N31" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>17.533196440793976</v>
       </c>
       <c r="O31" s="10">
@@ -3125,13 +3136,13 @@
       <c r="I32" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J32" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K32" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J32" s="7">
+        <f t="shared" si="2"/>
+        <v>9339</v>
+      </c>
+      <c r="K32" s="8">
+        <f t="shared" si="0"/>
+        <v>25.568788501026695</v>
       </c>
       <c r="L32" s="7">
         <v>78.11</v>
@@ -3140,7 +3151,7 @@
         <v>9080</v>
       </c>
       <c r="N32" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.859685147159478</v>
       </c>
       <c r="O32" s="10">
@@ -3184,13 +3195,13 @@
       <c r="I33" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J33" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K33" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J33" s="7">
+        <f t="shared" si="2"/>
+        <v>10909</v>
+      </c>
+      <c r="K33" s="8">
+        <f t="shared" si="0"/>
+        <v>29.867214236824093</v>
       </c>
       <c r="L33" s="7">
         <v>93.76</v>
@@ -3199,7 +3210,7 @@
         <v>10229</v>
       </c>
       <c r="N33" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.005475701574266</v>
       </c>
       <c r="O33" s="10">
@@ -3243,13 +3254,13 @@
       <c r="I34" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J34" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K34" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J34" s="7">
+        <f t="shared" si="2"/>
+        <v>10308</v>
+      </c>
+      <c r="K34" s="8">
+        <f t="shared" si="0"/>
+        <v>28.2217659137577</v>
       </c>
       <c r="L34" s="7">
         <v>89.06</v>
@@ -3258,7 +3269,7 @@
         <v>9181</v>
       </c>
       <c r="N34" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.136208076659823</v>
       </c>
       <c r="O34" s="10">
@@ -3302,13 +3313,13 @@
       <c r="I35" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J35" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K35" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J35" s="7">
+        <f t="shared" si="2"/>
+        <v>10869</v>
+      </c>
+      <c r="K35" s="8">
+        <f t="shared" si="0"/>
+        <v>29.757700205338811</v>
       </c>
       <c r="L35" s="7">
         <v>95.79</v>
@@ -3317,7 +3328,7 @@
         <v>10409</v>
       </c>
       <c r="N35" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.498288843258042</v>
       </c>
       <c r="O35" s="10">
@@ -3361,13 +3372,13 @@
       <c r="I36" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J36" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K36" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J36" s="7">
+        <f t="shared" si="2"/>
+        <v>10755</v>
+      </c>
+      <c r="K36" s="8">
+        <f t="shared" si="0"/>
+        <v>29.44558521560575</v>
       </c>
       <c r="L36" s="7">
         <v>91.66</v>
@@ -3376,7 +3387,7 @@
         <v>9859</v>
       </c>
       <c r="N36" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.992470910335388</v>
       </c>
       <c r="O36" s="10">
@@ -3420,13 +3431,13 @@
       <c r="I37" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J37" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K37" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J37" s="7">
+        <f t="shared" si="2"/>
+        <v>8628</v>
+      </c>
+      <c r="K37" s="8">
+        <f t="shared" si="0"/>
+        <v>23.622176591375769</v>
       </c>
       <c r="L37" s="7">
         <v>89.16</v>
@@ -3435,7 +3446,7 @@
         <v>7693</v>
       </c>
       <c r="N37" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.062286105407257</v>
       </c>
       <c r="O37" s="10">
@@ -3479,13 +3490,13 @@
       <c r="I38" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J38" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K38" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J38" s="7">
+        <f t="shared" si="2"/>
+        <v>10176</v>
+      </c>
+      <c r="K38" s="8">
+        <f t="shared" si="0"/>
+        <v>27.860369609856264</v>
       </c>
       <c r="L38" s="7">
         <v>79.58</v>
@@ -3494,7 +3505,7 @@
         <v>7812</v>
       </c>
       <c r="N38" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.388090349075977</v>
       </c>
       <c r="O38" s="10">
@@ -3538,13 +3549,13 @@
       <c r="I39" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J39" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K39" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J39" s="7">
+        <f t="shared" si="2"/>
+        <v>10649</v>
+      </c>
+      <c r="K39" s="8">
+        <f t="shared" si="0"/>
+        <v>29.155373032169745</v>
       </c>
       <c r="L39" s="7">
         <v>72.14</v>
@@ -3553,7 +3564,7 @@
         <v>7679</v>
       </c>
       <c r="N39" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.023956194387406</v>
       </c>
       <c r="O39" s="10">
@@ -3597,13 +3608,13 @@
       <c r="I40" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="J40" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K40" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J40" s="7">
+        <f t="shared" si="2"/>
+        <v>10155</v>
+      </c>
+      <c r="K40" s="8">
+        <f t="shared" si="0"/>
+        <v>27.802874743326488</v>
       </c>
       <c r="L40" s="7">
         <v>88.12</v>
@@ -3612,7 +3623,7 @@
         <v>8949</v>
       </c>
       <c r="N40" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.501026694045173</v>
       </c>
       <c r="O40" s="10">
@@ -3656,13 +3667,13 @@
       <c r="I41" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J41" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K41" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J41" s="7">
+        <f t="shared" si="2"/>
+        <v>9465</v>
+      </c>
+      <c r="K41" s="8">
+        <f t="shared" si="0"/>
+        <v>25.913757700205338</v>
       </c>
       <c r="L41" s="7">
         <v>93.04</v>
@@ -3671,7 +3682,7 @@
         <v>8799</v>
       </c>
       <c r="N41" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.090349075975361</v>
       </c>
       <c r="O41" s="10">
@@ -3715,13 +3726,13 @@
       <c r="I42" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J42" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K42" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J42" s="7">
+        <f t="shared" si="2"/>
+        <v>10384</v>
+      </c>
+      <c r="K42" s="8">
+        <f t="shared" si="0"/>
+        <v>28.429842573579741</v>
       </c>
       <c r="L42" s="7">
         <v>95.41</v>
@@ -3730,7 +3741,7 @@
         <v>9908</v>
       </c>
       <c r="N42" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.126625598904859</v>
       </c>
       <c r="O42" s="10">
@@ -3774,13 +3785,13 @@
       <c r="I43" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J43" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K43" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J43" s="7">
+        <f t="shared" si="2"/>
+        <v>11387</v>
+      </c>
+      <c r="K43" s="8">
+        <f t="shared" si="0"/>
+        <v>31.175906913073238</v>
       </c>
       <c r="L43" s="7">
         <v>90.85</v>
@@ -3789,7 +3800,7 @@
         <v>10096</v>
       </c>
       <c r="N43" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.641341546885695</v>
       </c>
       <c r="O43" s="10">
@@ -3833,13 +3844,13 @@
       <c r="I44" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J44" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K44" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J44" s="7">
+        <f t="shared" si="2"/>
+        <v>9034</v>
+      </c>
+      <c r="K44" s="8">
+        <f t="shared" si="0"/>
+        <v>24.733744010951405</v>
       </c>
       <c r="L44" s="7">
         <v>91.74</v>
@@ -3848,7 +3859,7 @@
         <v>8284</v>
       </c>
       <c r="N44" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>22.680355920602327</v>
       </c>
       <c r="O44" s="10">
@@ -3892,13 +3903,13 @@
       <c r="I45" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J45" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K45" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J45" s="7">
+        <f t="shared" si="2"/>
+        <v>11118</v>
+      </c>
+      <c r="K45" s="8">
+        <f t="shared" si="0"/>
+        <v>30.439425051334702</v>
       </c>
       <c r="L45" s="7">
         <v>77.88</v>
@@ -3907,7 +3918,7 @@
         <v>8653</v>
       </c>
       <c r="N45" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>23.690622861054074</v>
       </c>
       <c r="O45" s="10">
@@ -3951,13 +3962,13 @@
       <c r="I46" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J46" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K46" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J46" s="7">
+        <f t="shared" si="2"/>
+        <v>9916</v>
+      </c>
+      <c r="K46" s="8">
+        <f t="shared" si="0"/>
+        <v>27.148528405201915</v>
       </c>
       <c r="L46" s="7">
         <v>83.95</v>
@@ -3966,7 +3977,7 @@
         <v>8314</v>
       </c>
       <c r="N46" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>22.762491444216291</v>
       </c>
       <c r="O46" s="10">
@@ -4010,13 +4021,13 @@
       <c r="I47" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J47" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K47" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J47" s="7">
+        <f t="shared" si="2"/>
+        <v>7547</v>
+      </c>
+      <c r="K47" s="8">
+        <f t="shared" si="0"/>
+        <v>20.662559890485969</v>
       </c>
       <c r="L47" s="7">
         <v>89.9</v>
@@ -4025,7 +4036,7 @@
         <v>6775</v>
       </c>
       <c r="N47" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>18.548939082819988</v>
       </c>
       <c r="O47" s="10">
@@ -4069,13 +4080,13 @@
       <c r="I48" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J48" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K48" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J48" s="7">
+        <f t="shared" si="2"/>
+        <v>9550</v>
+      </c>
+      <c r="K48" s="8">
+        <f t="shared" si="0"/>
+        <v>26.146475017111566</v>
       </c>
       <c r="L48" s="7">
         <v>85.57</v>
@@ -4084,7 +4095,7 @@
         <v>8173</v>
       </c>
       <c r="N48" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>22.376454483230663</v>
       </c>
       <c r="O48" s="10">
@@ -4128,13 +4139,13 @@
       <c r="I49" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J49" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K49" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J49" s="7">
+        <f t="shared" si="2"/>
+        <v>6992</v>
+      </c>
+      <c r="K49" s="8">
+        <f t="shared" si="0"/>
+        <v>19.143052703627653</v>
       </c>
       <c r="L49" s="7">
         <v>83.12</v>
@@ -4143,7 +4154,7 @@
         <v>5723</v>
       </c>
       <c r="N49" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>15.668720054757015</v>
       </c>
       <c r="O49" s="10">
@@ -4187,13 +4198,13 @@
       <c r="I50" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J50" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K50" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J50" s="7">
+        <f t="shared" si="2"/>
+        <v>6346</v>
+      </c>
+      <c r="K50" s="8">
+        <f t="shared" si="0"/>
+        <v>17.374401095140314</v>
       </c>
       <c r="L50" s="7">
         <v>91.84</v>
@@ -4202,7 +4213,7 @@
         <v>5559</v>
       </c>
       <c r="N50" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>15.219712525667351</v>
       </c>
       <c r="O50" s="10">
@@ -4246,13 +4257,13 @@
       <c r="I51" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J51" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K51" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J51" s="7">
+        <f t="shared" si="2"/>
+        <v>9440</v>
+      </c>
+      <c r="K51" s="8">
+        <f t="shared" si="0"/>
+        <v>25.845311430527037</v>
       </c>
       <c r="L51" s="7">
         <v>85.98</v>
@@ -4261,7 +4272,7 @@
         <v>8016</v>
       </c>
       <c r="N51" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>21.946611909650922</v>
       </c>
       <c r="O51" s="10">
@@ -4305,13 +4316,13 @@
       <c r="I52" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J52" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K52" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J52" s="7">
+        <f t="shared" si="2"/>
+        <v>7250</v>
+      </c>
+      <c r="K52" s="8">
+        <f t="shared" si="0"/>
+        <v>19.849418206707735</v>
       </c>
       <c r="L52" s="7">
         <v>93.38</v>
@@ -4320,7 +4331,7 @@
         <v>5652</v>
       </c>
       <c r="N52" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>15.474332648870636</v>
       </c>
       <c r="O52" s="10">
@@ -4364,13 +4375,13 @@
       <c r="I53" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J53" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K53" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J53" s="7">
+        <f t="shared" si="2"/>
+        <v>8658</v>
+      </c>
+      <c r="K53" s="8">
+        <f t="shared" si="0"/>
+        <v>23.704312114989733</v>
       </c>
       <c r="L53" s="7">
         <v>85.92</v>
@@ -4379,7 +4390,7 @@
         <v>7174</v>
       </c>
       <c r="N53" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>19.641341546885695</v>
       </c>
       <c r="O53" s="10">
@@ -4423,13 +4434,13 @@
       <c r="I54" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J54" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K54" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J54" s="7">
+        <f t="shared" si="2"/>
+        <v>10518</v>
+      </c>
+      <c r="K54" s="8">
+        <f t="shared" si="0"/>
+        <v>28.79671457905544</v>
       </c>
       <c r="L54" s="7">
         <v>83.76</v>
@@ -4438,7 +4449,7 @@
         <v>8808</v>
       </c>
       <c r="N54" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.114989733059549</v>
       </c>
       <c r="O54" s="10">
@@ -4482,13 +4493,13 @@
       <c r="I55" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J55" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K55" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J55" s="7">
+        <f t="shared" si="2"/>
+        <v>9756</v>
+      </c>
+      <c r="K55" s="8">
+        <f t="shared" si="0"/>
+        <v>26.710472279260781</v>
       </c>
       <c r="L55" s="7">
         <v>92.2</v>
@@ -4497,7 +4508,7 @@
         <v>8996</v>
       </c>
       <c r="N55" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.629705681040384</v>
       </c>
       <c r="O55" s="10">
@@ -4541,13 +4552,13 @@
       <c r="I56" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="J56" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K56" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J56" s="7">
+        <f t="shared" si="2"/>
+        <v>7209</v>
+      </c>
+      <c r="K56" s="8">
+        <f t="shared" si="0"/>
+        <v>19.737166324435318</v>
       </c>
       <c r="L56" s="7">
         <v>92.53</v>
@@ -4556,7 +4567,7 @@
         <v>5601</v>
       </c>
       <c r="N56" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>15.3347022587269</v>
       </c>
       <c r="O56" s="10">
@@ -4600,13 +4611,13 @@
       <c r="I57" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="J57" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K57" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J57" s="7">
+        <f t="shared" si="2"/>
+        <v>11288</v>
+      </c>
+      <c r="K57" s="8">
+        <f t="shared" si="0"/>
+        <v>30.904859685147159</v>
       </c>
       <c r="L57" s="7">
         <v>73.900000000000006</v>
@@ -4615,7 +4626,7 @@
         <v>7527</v>
       </c>
       <c r="N57" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>20.607802874743328</v>
       </c>
       <c r="O57" s="10">
@@ -4659,13 +4670,13 @@
       <c r="I58" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="J58" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K58" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J58" s="7">
+        <f t="shared" si="2"/>
+        <v>9806</v>
+      </c>
+      <c r="K58" s="8">
+        <f t="shared" si="0"/>
+        <v>26.847364818617386</v>
       </c>
       <c r="L58" s="7">
         <v>93.91</v>
@@ -4674,7 +4685,7 @@
         <v>9210</v>
       </c>
       <c r="N58" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.215605749486652</v>
       </c>
       <c r="O58" s="10">
@@ -4718,13 +4729,13 @@
       <c r="I59" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="J59" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K59" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J59" s="7">
+        <f t="shared" si="2"/>
+        <v>7746</v>
+      </c>
+      <c r="K59" s="8">
+        <f t="shared" si="0"/>
+        <v>21.207392197125255</v>
       </c>
       <c r="L59" s="7">
         <v>97.56</v>
@@ -4733,7 +4744,7 @@
         <v>7557</v>
       </c>
       <c r="N59" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>20.689938398357288</v>
       </c>
       <c r="O59" s="10">
@@ -4777,13 +4788,13 @@
       <c r="I60" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="J60" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K60" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J60" s="7">
+        <f t="shared" si="2"/>
+        <v>7772</v>
+      </c>
+      <c r="K60" s="8">
+        <f t="shared" si="0"/>
+        <v>21.278576317590691</v>
       </c>
       <c r="L60" s="7">
         <v>97.23</v>
@@ -4792,7 +4803,7 @@
         <v>7553</v>
       </c>
       <c r="N60" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>20.67898699520876</v>
       </c>
       <c r="O60" s="10">
@@ -4836,13 +4847,13 @@
       <c r="I61" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="J61" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K61" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J61" s="7">
+        <f t="shared" si="2"/>
+        <v>6960</v>
+      </c>
+      <c r="K61" s="8">
+        <f t="shared" si="0"/>
+        <v>19.055441478439427</v>
       </c>
       <c r="L61" s="7">
         <v>99.51</v>
@@ -4851,7 +4862,7 @@
         <v>6919</v>
       </c>
       <c r="N61" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>18.943189596167009</v>
       </c>
       <c r="O61" s="10">
@@ -4895,13 +4906,13 @@
       <c r="I62" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="J62" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K62" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J62" s="7">
+        <f t="shared" si="2"/>
+        <v>6723</v>
+      </c>
+      <c r="K62" s="8">
+        <f t="shared" si="0"/>
+        <v>18.406570841889117</v>
       </c>
       <c r="L62" s="7">
         <v>95.37</v>
@@ -4910,7 +4921,7 @@
         <v>6409</v>
       </c>
       <c r="N62" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>17.546885694729639</v>
       </c>
       <c r="O62" s="10">
@@ -4954,13 +4965,13 @@
       <c r="I63" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="J63" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K63" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J63" s="7">
+        <f t="shared" si="2"/>
+        <v>7824</v>
+      </c>
+      <c r="K63" s="8">
+        <f t="shared" si="0"/>
+        <v>21.420944558521562</v>
       </c>
       <c r="L63" s="7">
         <v>92.6</v>
@@ -4969,7 +4980,7 @@
         <v>7245</v>
       </c>
       <c r="N63" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>19.835728952772072</v>
       </c>
       <c r="O63" s="10">
@@ -5013,13 +5024,13 @@
       <c r="I64" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J64" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K64" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J64" s="7">
+        <f t="shared" si="2"/>
+        <v>10406</v>
+      </c>
+      <c r="K64" s="8">
+        <f t="shared" si="0"/>
+        <v>28.490075290896645</v>
       </c>
       <c r="L64" s="7">
         <v>88.9</v>
@@ -5028,7 +5039,7 @@
         <v>9250</v>
       </c>
       <c r="N64" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.325119780971939</v>
       </c>
       <c r="O64" s="10">
@@ -5072,13 +5083,13 @@
       <c r="I65" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J65" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K65" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J65" s="7">
+        <f t="shared" si="2"/>
+        <v>10753</v>
+      </c>
+      <c r="K65" s="8">
+        <f t="shared" si="0"/>
+        <v>29.440109514031484</v>
       </c>
       <c r="L65" s="7">
         <v>84.02</v>
@@ -5087,7 +5098,7 @@
         <v>9035</v>
       </c>
       <c r="N65" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.736481861738536</v>
       </c>
       <c r="O65" s="10">
@@ -5131,13 +5142,13 @@
       <c r="I66" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J66" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K66" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J66" s="7">
+        <f t="shared" si="2"/>
+        <v>10794</v>
+      </c>
+      <c r="K66" s="8">
+        <f t="shared" si="0"/>
+        <v>29.552361396303901</v>
       </c>
       <c r="L66" s="7">
         <v>95.19</v>
@@ -5146,7 +5157,7 @@
         <v>10276</v>
       </c>
       <c r="N66" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.134154688569474</v>
       </c>
       <c r="O66" s="17"/>
@@ -5182,13 +5193,13 @@
       <c r="I67" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J67" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K67" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J67" s="7">
+        <f t="shared" ref="J67:J96" si="3">_xlfn.DAYS(F67,E67)</f>
+        <v>10802</v>
+      </c>
+      <c r="K67" s="8">
+        <f t="shared" si="0"/>
+        <v>29.574264202600958</v>
       </c>
       <c r="L67" s="7">
         <v>91.12</v>
@@ -5197,7 +5208,7 @@
         <v>9843</v>
       </c>
       <c r="N67" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.948665297741272</v>
       </c>
       <c r="O67" s="10">
@@ -5241,13 +5252,13 @@
       <c r="I68" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J68" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K68" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J68" s="7">
+        <f t="shared" si="3"/>
+        <v>10799</v>
+      </c>
+      <c r="K68" s="8">
+        <f t="shared" si="0"/>
+        <v>29.566050650239561</v>
       </c>
       <c r="L68" s="7">
         <v>98.45</v>
@@ -5256,7 +5267,7 @@
         <v>10632</v>
       </c>
       <c r="N68" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>29.108829568788501</v>
       </c>
       <c r="O68" s="17"/>
@@ -5292,13 +5303,13 @@
       <c r="I69" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J69" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K69" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J69" s="7">
+        <f t="shared" si="3"/>
+        <v>10786</v>
+      </c>
+      <c r="K69" s="8">
+        <f t="shared" si="0"/>
+        <v>29.530458590006845</v>
       </c>
       <c r="L69" s="7">
         <v>96.74</v>
@@ -5307,7 +5318,7 @@
         <v>10434</v>
       </c>
       <c r="N69" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.566735112936346</v>
       </c>
       <c r="O69" s="17"/>
@@ -5343,13 +5354,13 @@
       <c r="I70" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J70" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K70" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J70" s="7">
+        <f t="shared" si="3"/>
+        <v>10786</v>
+      </c>
+      <c r="K70" s="8">
+        <f t="shared" si="0"/>
+        <v>29.530458590006845</v>
       </c>
       <c r="L70" s="7">
         <v>82.64</v>
@@ -5358,7 +5369,7 @@
         <v>8914</v>
       </c>
       <c r="N70" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.40520191649555</v>
       </c>
       <c r="O70" s="10">
@@ -5402,13 +5413,13 @@
       <c r="I71" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J71" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K71" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J71" s="7">
+        <f t="shared" si="3"/>
+        <v>10386</v>
+      </c>
+      <c r="K71" s="8">
+        <f t="shared" si="0"/>
+        <v>28.435318275154003</v>
       </c>
       <c r="L71" s="7">
         <v>96.93</v>
@@ -5417,7 +5428,7 @@
         <v>9786</v>
       </c>
       <c r="N71" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.792607802874745</v>
       </c>
       <c r="O71" s="10">
@@ -5461,13 +5472,13 @@
       <c r="I72" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="J72" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K72" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J72" s="7">
+        <f t="shared" si="3"/>
+        <v>10791</v>
+      </c>
+      <c r="K72" s="8">
+        <f t="shared" si="0"/>
+        <v>29.544147843942504</v>
       </c>
       <c r="L72" s="7">
         <v>89.34</v>
@@ -5476,7 +5487,7 @@
         <v>9642</v>
       </c>
       <c r="N72" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.39835728952772</v>
       </c>
       <c r="O72" s="10">
@@ -5520,13 +5531,13 @@
       <c r="I73" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J73" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K73" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J73" s="7">
+        <f t="shared" si="3"/>
+        <v>11603</v>
+      </c>
+      <c r="K73" s="8">
+        <f t="shared" si="0"/>
+        <v>31.767282683093772</v>
       </c>
       <c r="L73" s="7">
         <v>92.97</v>
@@ -5535,7 +5546,7 @@
         <v>10788</v>
       </c>
       <c r="N73" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>29.535934291581111</v>
       </c>
       <c r="O73" s="17"/>
@@ -5571,13 +5582,13 @@
       <c r="I74" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J74" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K74" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J74" s="7">
+        <f t="shared" si="3"/>
+        <v>9785</v>
+      </c>
+      <c r="K74" s="8">
+        <f t="shared" si="0"/>
+        <v>26.78986995208761</v>
       </c>
       <c r="L74" s="7">
         <v>95.4</v>
@@ -5586,7 +5597,7 @@
         <v>9333</v>
       </c>
       <c r="N74" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.552361396303901</v>
       </c>
       <c r="O74" s="10">
@@ -5630,13 +5641,13 @@
       <c r="I75" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J75" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K75" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J75" s="7">
+        <f t="shared" si="3"/>
+        <v>10859</v>
+      </c>
+      <c r="K75" s="8">
+        <f t="shared" si="0"/>
+        <v>29.730321697467488</v>
       </c>
       <c r="L75" s="7">
         <v>99.17</v>
@@ -5645,7 +5656,7 @@
         <v>10770</v>
       </c>
       <c r="N75" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>29.486652977412732</v>
       </c>
       <c r="O75" s="10">
@@ -5689,13 +5700,13 @@
       <c r="I76" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J76" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K76" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J76" s="7">
+        <f t="shared" si="3"/>
+        <v>11741</v>
+      </c>
+      <c r="K76" s="8">
+        <f t="shared" si="0"/>
+        <v>32.145106091717999</v>
       </c>
       <c r="L76" s="7">
         <v>98.56</v>
@@ -5704,7 +5715,7 @@
         <v>9722</v>
       </c>
       <c r="N76" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.617385352498289</v>
       </c>
       <c r="O76" s="10">
@@ -5748,13 +5759,13 @@
       <c r="I77" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J77" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K77" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J77" s="7">
+        <f t="shared" si="3"/>
+        <v>10023</v>
+      </c>
+      <c r="K77" s="8">
+        <f t="shared" si="0"/>
+        <v>27.441478439425051</v>
       </c>
       <c r="L77" s="7">
         <v>97.43</v>
@@ -5763,7 +5774,7 @@
         <v>9763</v>
       </c>
       <c r="N77" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.729637234770706</v>
       </c>
       <c r="O77" s="10">
@@ -5807,13 +5818,13 @@
       <c r="I78" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J78" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K78" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J78" s="7">
+        <f t="shared" si="3"/>
+        <v>10765</v>
+      </c>
+      <c r="K78" s="8">
+        <f t="shared" si="0"/>
+        <v>29.472963723477072</v>
       </c>
       <c r="L78" s="7">
         <v>89.52</v>
@@ -5822,7 +5833,7 @@
         <v>9637</v>
       </c>
       <c r="N78" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.38466803559206</v>
       </c>
       <c r="O78" s="10">
@@ -5866,13 +5877,13 @@
       <c r="I79" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J79" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K79" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J79" s="7">
+        <f t="shared" si="3"/>
+        <v>11625</v>
+      </c>
+      <c r="K79" s="8">
+        <f t="shared" si="0"/>
+        <v>31.827515400410679</v>
       </c>
       <c r="L79" s="7">
         <v>81.650000000000006</v>
@@ -5881,7 +5892,7 @@
         <v>9175</v>
       </c>
       <c r="N79" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.119780971937029</v>
       </c>
       <c r="O79" s="10">
@@ -5925,13 +5936,13 @@
       <c r="I80" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J80" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K80" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J80" s="7">
+        <f t="shared" si="3"/>
+        <v>11054</v>
+      </c>
+      <c r="K80" s="8">
+        <f t="shared" si="0"/>
+        <v>30.264202600958249</v>
       </c>
       <c r="L80" s="7">
         <v>89.65</v>
@@ -5940,7 +5951,7 @@
         <v>9911</v>
       </c>
       <c r="N80" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.134839151266256</v>
       </c>
       <c r="O80" s="10">
@@ -5984,13 +5995,13 @@
       <c r="I81" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J81" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K81" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J81" s="7">
+        <f t="shared" si="3"/>
+        <v>11057</v>
+      </c>
+      <c r="K81" s="8">
+        <f t="shared" si="0"/>
+        <v>30.272416153319643</v>
       </c>
       <c r="L81" s="7">
         <v>80.430000000000007</v>
@@ -5999,7 +6010,7 @@
         <v>8894</v>
       </c>
       <c r="N81" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.350444900752908</v>
       </c>
       <c r="O81" s="10">
@@ -6043,13 +6054,13 @@
       <c r="I82" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J82" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K82" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J82" s="7">
+        <f t="shared" si="3"/>
+        <v>11059</v>
+      </c>
+      <c r="K82" s="8">
+        <f t="shared" si="0"/>
+        <v>30.277891854893909</v>
       </c>
       <c r="L82" s="7">
         <v>95.57</v>
@@ -6058,7 +6069,7 @@
         <v>10570</v>
       </c>
       <c r="N82" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.939082819986311</v>
       </c>
       <c r="O82" s="10">
@@ -6102,13 +6113,13 @@
       <c r="I83" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J83" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K83" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J83" s="7">
+        <f t="shared" si="3"/>
+        <v>11055</v>
+      </c>
+      <c r="K83" s="8">
+        <f t="shared" si="0"/>
+        <v>30.266940451745381</v>
       </c>
       <c r="L83" s="7">
         <v>93</v>
@@ -6117,7 +6128,7 @@
         <v>10282</v>
       </c>
       <c r="N83" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.150581793292265</v>
       </c>
       <c r="O83" s="10">
@@ -6161,13 +6172,13 @@
       <c r="I84" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="J84" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K84" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J84" s="7">
+        <f t="shared" si="3"/>
+        <v>11061</v>
+      </c>
+      <c r="K84" s="8">
+        <f t="shared" si="0"/>
+        <v>30.283367556468171</v>
       </c>
       <c r="L84" s="7">
         <v>95.27</v>
@@ -6176,7 +6187,7 @@
         <v>10539</v>
       </c>
       <c r="N84" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.854209445585216</v>
       </c>
       <c r="O84" s="10">
@@ -6220,13 +6231,13 @@
       <c r="I85" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J85" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K85" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J85" s="7">
+        <f t="shared" si="3"/>
+        <v>11066</v>
+      </c>
+      <c r="K85" s="8">
+        <f t="shared" si="0"/>
+        <v>30.297056810403834</v>
       </c>
       <c r="L85" s="7">
         <v>96.89</v>
@@ -6235,7 +6246,7 @@
         <v>10723</v>
       </c>
       <c r="N85" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>29.357973990417523</v>
       </c>
       <c r="O85" s="10">
@@ -6279,13 +6290,13 @@
       <c r="I86" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J86" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K86" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J86" s="7">
+        <f t="shared" si="3"/>
+        <v>10344</v>
+      </c>
+      <c r="K86" s="8">
+        <f t="shared" si="0"/>
+        <v>28.320328542094455</v>
       </c>
       <c r="L86" s="7">
         <v>85.79</v>
@@ -6294,7 +6305,7 @@
         <v>8874</v>
       </c>
       <c r="N86" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>24.295687885010267</v>
       </c>
       <c r="O86" s="10">
@@ -6338,13 +6349,13 @@
       <c r="I87" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J87" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K87" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J87" s="7">
+        <f t="shared" si="3"/>
+        <v>11078</v>
+      </c>
+      <c r="K87" s="8">
+        <f t="shared" si="0"/>
+        <v>30.329911019849419</v>
       </c>
       <c r="L87" s="7">
         <v>96.16</v>
@@ -6353,7 +6364,7 @@
         <v>10638</v>
       </c>
       <c r="N87" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>29.125256673511295</v>
       </c>
       <c r="O87" s="10">
@@ -6397,13 +6408,13 @@
       <c r="I88" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J88" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K88" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J88" s="7">
+        <f t="shared" si="3"/>
+        <v>11066</v>
+      </c>
+      <c r="K88" s="8">
+        <f t="shared" si="0"/>
+        <v>30.297056810403834</v>
       </c>
       <c r="L88" s="7">
         <v>93.26</v>
@@ -6412,7 +6423,7 @@
         <v>10321</v>
       </c>
       <c r="N88" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.257357973990416</v>
       </c>
       <c r="O88" s="10">
@@ -6456,13 +6467,13 @@
       <c r="I89" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J89" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K89" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J89" s="7">
+        <f t="shared" si="3"/>
+        <v>11075</v>
+      </c>
+      <c r="K89" s="8">
+        <f t="shared" si="0"/>
+        <v>30.321697467488022</v>
       </c>
       <c r="L89" s="7">
         <v>93.9</v>
@@ -6471,7 +6482,7 @@
         <v>10399</v>
       </c>
       <c r="N89" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.470910335386723</v>
       </c>
       <c r="O89" s="10">
@@ -6515,13 +6526,13 @@
       <c r="I90" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J90" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K90" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J90" s="7">
+        <f t="shared" si="3"/>
+        <v>10643</v>
+      </c>
+      <c r="K90" s="8">
+        <f t="shared" si="0"/>
+        <v>29.138945927446954</v>
       </c>
       <c r="L90" s="7">
         <v>85.81</v>
@@ -6530,7 +6541,7 @@
         <v>9134</v>
       </c>
       <c r="N90" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>25.007529089664612</v>
       </c>
       <c r="O90" s="17"/>
@@ -6566,13 +6577,13 @@
       <c r="I91" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="J91" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K91" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J91" s="7">
+        <f t="shared" si="3"/>
+        <v>11082</v>
+      </c>
+      <c r="K91" s="8">
+        <f t="shared" si="0"/>
+        <v>30.340862422997947</v>
       </c>
       <c r="L91" s="7">
         <v>92.62</v>
@@ -6581,7 +6592,7 @@
         <v>10264</v>
       </c>
       <c r="N91" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>28.101300479123889</v>
       </c>
       <c r="O91" s="10">
@@ -6625,13 +6636,13 @@
       <c r="I92" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J92" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K92" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J92" s="7">
+        <f t="shared" si="3"/>
+        <v>10928</v>
+      </c>
+      <c r="K92" s="8">
+        <f t="shared" si="0"/>
+        <v>29.919233401779604</v>
       </c>
       <c r="L92" s="7">
         <v>91.25</v>
@@ -6640,7 +6651,7 @@
         <v>9972</v>
       </c>
       <c r="N92" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>27.301848049281315</v>
       </c>
       <c r="O92" s="10">
@@ -6684,13 +6695,13 @@
       <c r="I93" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J93" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K93" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J93" s="7">
+        <f t="shared" si="3"/>
+        <v>10918</v>
+      </c>
+      <c r="K93" s="8">
+        <f t="shared" si="0"/>
+        <v>29.891854893908281</v>
       </c>
       <c r="L93" s="7">
         <v>89.74</v>
@@ -6699,7 +6710,7 @@
         <v>9799</v>
       </c>
       <c r="N93" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.828199863107461</v>
       </c>
       <c r="O93" s="10">
@@ -6743,13 +6754,13 @@
       <c r="I94" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J94" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K94" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J94" s="7">
+        <f t="shared" si="3"/>
+        <v>10946</v>
+      </c>
+      <c r="K94" s="8">
+        <f t="shared" si="0"/>
+        <v>29.968514715947983</v>
       </c>
       <c r="L94" s="7">
         <v>87.33</v>
@@ -6758,7 +6769,7 @@
         <v>9559</v>
       </c>
       <c r="N94" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.171115674195757</v>
       </c>
       <c r="O94" s="17"/>
@@ -6794,13 +6805,13 @@
       <c r="I95" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J95" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K95" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J95" s="7">
+        <f t="shared" si="3"/>
+        <v>10876</v>
+      </c>
+      <c r="K95" s="8">
+        <f t="shared" si="0"/>
+        <v>29.776865160848732</v>
       </c>
       <c r="L95" s="7">
         <v>87.79</v>
@@ -6809,7 +6820,7 @@
         <v>9546</v>
       </c>
       <c r="N95" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.135523613963038</v>
       </c>
       <c r="O95" s="10">
@@ -6853,13 +6864,13 @@
       <c r="I96" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="J96" s="7" t="e">
-        <f t="shared" ca="1" si="0"/>
-        <v>#NAME?</v>
-      </c>
-      <c r="K96" s="8" t="e">
-        <f t="shared" ca="1" si="1"/>
-        <v>#NAME?</v>
+      <c r="J96" s="7">
+        <f t="shared" si="3"/>
+        <v>10887</v>
+      </c>
+      <c r="K96" s="8">
+        <f t="shared" si="0"/>
+        <v>29.806981519507186</v>
       </c>
       <c r="L96" s="7">
         <v>87.89</v>
@@ -6868,7 +6879,7 @@
         <v>9570</v>
       </c>
       <c r="N96" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>26.201232032854211</v>
       </c>
       <c r="O96" s="10">
@@ -12665,7 +12676,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12828,8 +12839,17 @@
         <v>211</v>
       </c>
     </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="41" t="s">
+        <v>273</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>274</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>